<commit_message>
Tela de perfil de Trabalhador e Contratante
</commit_message>
<xml_diff>
--- a/Docs/Testes/Casos de Teste.xlsx
+++ b/Docs/Testes/Casos de Teste.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\josue.rosario\Documents\Projeto_Base\Docs\Testes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aluno\Documents\Iscaro👀\Josue\projeto-conclusao-ibico\Docs\Testes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89EE332B-FA9E-4B69-AC97-7E879A8C9102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF70FAC3-0923-47AE-B6EF-628968BC79EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B39D3B3E-C0E7-4FBE-A703-F38F16FF52B7}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{B39D3B3E-C0E7-4FBE-A703-F38F16FF52B7}"/>
   </bookViews>
   <sheets>
     <sheet name="RESULTADOS" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="49">
   <si>
     <t>ID</t>
   </si>
@@ -117,9 +117,6 @@
     <t>Ao inserir um usuário e senha corretos o sistema deve levar a tela inicial</t>
   </si>
   <si>
-    <t>Usuarío deve estar cadastrado no banco</t>
-  </si>
-  <si>
     <t>Usuario: josedasilva
 senha: 1234</t>
   </si>
@@ -127,45 +124,82 @@
     <t>COMO EXECUTAR O TESTE</t>
   </si>
   <si>
+    <t>PASSOU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">createExemplo() deve cadastrar um exemplo </t>
+  </si>
+  <si>
+    <t>TESTES IMPLEMENTADOS</t>
+  </si>
+  <si>
+    <t>DESCRIÇÃO</t>
+  </si>
+  <si>
+    <t>UNITÁRIOS</t>
+  </si>
+  <si>
+    <t>FUNCIONAIS</t>
+  </si>
+  <si>
+    <t>TESTES QUE PASSARAM</t>
+  </si>
+  <si>
+    <t>TESTES QUE NÃO PASSARAM</t>
+  </si>
+  <si>
+    <t>TESTES NÃO IMPLEMENTADOS</t>
+  </si>
+  <si>
+    <t>SIM</t>
+  </si>
+  <si>
+    <t>NÃO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Abrir o sistema
+2. cadastrar usuario e senha
+</t>
+  </si>
+  <si>
+    <t>Cadastro</t>
+  </si>
+  <si>
+    <t>Ao inserir um usuário e senha corretos o sistema deve levar a tela de Login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10/11/2026
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Josué Rosario
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PASSOU
+</t>
+  </si>
+  <si>
+    <t>CTF-002</t>
+  </si>
+  <si>
+    <t>O usuário deve estar cadastrado no banco de dados</t>
+  </si>
+  <si>
     <t>1. Abrir o sistema
-2. Inserir usuário e senha válido e pressiona ok</t>
-  </si>
-  <si>
-    <t>1. A tela inicial foi mostrada
-2. O nome do usuário foi corretamente mostrado</t>
-  </si>
-  <si>
-    <t>PASSOU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">createExemplo() deve cadastrar um exemplo </t>
-  </si>
-  <si>
-    <t>TESTES IMPLEMENTADOS</t>
-  </si>
-  <si>
-    <t>DESCRIÇÃO</t>
-  </si>
-  <si>
-    <t>UNITÁRIOS</t>
-  </si>
-  <si>
-    <t>FUNCIONAIS</t>
-  </si>
-  <si>
-    <t>TESTES QUE PASSARAM</t>
-  </si>
-  <si>
-    <t>TESTES QUE NÃO PASSARAM</t>
-  </si>
-  <si>
-    <t>TESTES NÃO IMPLEMENTADOS</t>
-  </si>
-  <si>
-    <t>SIM</t>
-  </si>
-  <si>
-    <t>NÃO</t>
+2. cadastrar usuario e senha</t>
+  </si>
+  <si>
+    <t>1. A tela inicial foi mostrada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. O cpf é autentico
+2. O cpf não pode ser usado mais de uma vez
+3. O cpf deve conter apenas números
+4. Email do usuário
+5. Idade do usuário
+6. 
+</t>
   </si>
 </sst>
 </file>
@@ -239,7 +273,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -257,6 +291,25 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -590,30 +643,52 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="525" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{74F26EA1-E391-45FF-B518-653AF88DA29F}">
+  <we:reference id="WA200010215" version="2.0.0.0" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200010215" version="2.0.0.0" store="WA200010215" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="bps.codex_control.document_id" value="&quot;acd9fb40-3c08-4c02-a4a9-f8e987e018ce&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3844782C-A2B1-4136-86F8-0F29B8267B23}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="28.85546875" customWidth="1"/>
+    <col min="1" max="1" width="28.81640625" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="18.5703125" customWidth="1"/>
+    <col min="3" max="3" width="18.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C1" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="5" t="s">
         <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>38</v>
       </c>
       <c r="B2" s="7">
         <f>COUNTIFS(UNITARIOS!$E:$E,"=NÃO")</f>
@@ -621,12 +696,12 @@
       </c>
       <c r="C2" s="7">
         <f>COUNTIFS(FUNCIONAIS!$D:$D,"=NÃO")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B3" s="7">
         <f>COUNTIFS(UNITARIOS!$E:$E,"=SIM")</f>
@@ -637,9 +712,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B4" s="7">
         <f>COUNTIFS(UNITARIOS!M:M,"=PASSOU")</f>
@@ -647,12 +722,12 @@
       </c>
       <c r="C4" s="7">
         <f>COUNTIFS(FUNCIONAIS!$L:$L,"=PASSOU")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B5" s="7">
         <f>COUNTIFS(UNITARIOS!M:M,"=NAO PASSOU")</f>
@@ -671,24 +746,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33D0CAC7-316E-46CB-A569-E04FC4195B48}">
   <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="26.85546875" customWidth="1"/>
-    <col min="7" max="7" width="28.5703125" customWidth="1"/>
-    <col min="8" max="8" width="36.140625" customWidth="1"/>
-    <col min="9" max="9" width="60.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="43.140625" customWidth="1"/>
-    <col min="11" max="11" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="36.42578125" customWidth="1"/>
-    <col min="13" max="13" width="20.85546875" customWidth="1"/>
+    <col min="1" max="1" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="39.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.81640625" customWidth="1"/>
+    <col min="7" max="7" width="28.54296875" customWidth="1"/>
+    <col min="8" max="8" width="36.1796875" customWidth="1"/>
+    <col min="9" max="9" width="60.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="43.1796875" customWidth="1"/>
+    <col min="11" max="11" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="36.453125" customWidth="1"/>
+    <col min="13" max="13" width="20.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -729,7 +804,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:13" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -740,10 +815,10 @@
         <v>8</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>9</v>
@@ -764,7 +839,7 @@
         <v>18</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -775,95 +850,123 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C7A0F25-71DD-4BBC-9B61-33CCED0C99FF}">
-  <dimension ref="A1:L2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="66.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="47.7109375" customWidth="1"/>
-    <col min="6" max="6" width="35.7109375" customWidth="1"/>
-    <col min="7" max="7" width="60.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="66.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="47.7265625" customWidth="1"/>
+    <col min="6" max="6" width="35.7265625" customWidth="1"/>
+    <col min="7" max="7" width="60.7265625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="74" customWidth="1"/>
-    <col min="9" max="9" width="46.85546875" customWidth="1"/>
-    <col min="10" max="10" width="14.7109375" customWidth="1"/>
-    <col min="11" max="11" width="32.28515625" customWidth="1"/>
-    <col min="12" max="12" width="20.5703125" customWidth="1"/>
+    <col min="9" max="9" width="46.81640625" customWidth="1"/>
+    <col min="10" max="10" width="14.7265625" customWidth="1"/>
+    <col min="11" max="11" width="32.26953125" customWidth="1"/>
+    <col min="12" max="12" width="20.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="1" t="s">
+      <c r="G1" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:12" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" s="9"/>
+      <c r="F2" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="I2" s="9"/>
+      <c r="J2" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="K2" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="L2" s="14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="32.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C3" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="E2" s="2" t="s">
+      <c r="D3" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F3" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="I2" s="2"/>
-      <c r="J2" s="4">
-        <v>45971</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>30</v>
-      </c>
+      <c r="G3" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>